<commit_message>
feat: Implement Excel import functionality for business proposals, including parsing, aggregation, and database upsert.
</commit_message>
<xml_diff>
--- a/database/DefinicaoCampos.xlsx
+++ b/database/DefinicaoCampos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SuperCRM\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C2422E-B58C-4658-800B-7F94D9F2BEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D888ED14-0305-4552-8E9F-582A2284678B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7842B42A-80A9-4B36-ADEF-5A4F17B0DFD4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="48">
   <si>
     <t>Sheet</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Nome Coluna Português</t>
   </si>
   <si>
-    <t>Criar Coleção</t>
-  </si>
-  <si>
     <t>Grid 1</t>
   </si>
   <si>
@@ -59,9 +56,6 @@
     <t>Id da Proposta</t>
   </si>
   <si>
-    <t>Não</t>
-  </si>
-  <si>
     <t>Main Contract ID</t>
   </si>
   <si>
@@ -186,21 +180,6 @@
   </si>
   <si>
     <t>Currency</t>
-  </si>
-  <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>FunnelPercentage</t>
-  </si>
-  <si>
-    <t>ProposalStatus</t>
-  </si>
-  <si>
-    <t>AgingProposal</t>
-  </si>
-  <si>
-    <t>AgingStatus</t>
   </si>
 </sst>
 </file>
@@ -587,17 +566,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{726463BF-C24B-4C13-990F-3931E4B319DE}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
     <col min="3" max="3" width="27.7109375" customWidth="1"/>
     <col min="4" max="4" width="24.42578125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -608,401 +586,329 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="3" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="3" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="3" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
         <v>20</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C10" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="D10" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="D11" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>24</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="D12" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>26</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C13" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="D13" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
         <v>28</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C14" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="D14" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s">
         <v>30</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="D15" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" t="s">
         <v>32</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="D16" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" t="s">
         <v>34</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
         <v>36</v>
       </c>
-      <c r="C17" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C19" t="s">
         <v>37</v>
       </c>
-      <c r="C18" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="D19" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
         <v>38</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C20" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
         <v>40</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C22" t="s">
         <v>40</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="D22" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" t="s">
         <v>41</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C23" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="D23" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
         <v>42</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C24" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>4</v>
-      </c>
-      <c r="B23" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" t="s">
-        <v>44</v>
-      </c>
       <c r="D24" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>